<commit_message>
Day 19 is uploaded
</commit_message>
<xml_diff>
--- a/playwright/testdata/readexcel.xlsx
+++ b/playwright/testdata/readexcel.xlsx
@@ -1,33 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aryan Upadhyay\OneDrive\Desktop\projects\playwright\testdata\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E47FFBA-2585-4F80-AD32-736852A4A7F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Sheet2" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Sheet3" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Sheet4" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Sheet5" state="visible" r:id="rId8"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="32">
   <si>
     <t>afhasias</t>
   </si>
@@ -35,9 +26,15 @@
     <t>fnawkefnnask</t>
   </si>
   <si>
+    <t>f</t>
+  </si>
+  <si>
     <t>ergf</t>
   </si>
   <si>
+    <t>dfsa</t>
+  </si>
+  <si>
     <t>2rf</t>
   </si>
   <si>
@@ -47,10 +44,10 @@
     <t>sdf</t>
   </si>
   <si>
-    <t>dfsa</t>
-  </si>
-  <si>
-    <t>f</t>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>name</t>
   </si>
   <si>
     <t>email</t>
@@ -59,7 +56,7 @@
     <t>password</t>
   </si>
   <si>
-    <t>name</t>
+    <t>https://demoapps.qspiders.com/ui?scenario=1</t>
   </si>
   <si>
     <t>Aryan</t>
@@ -71,12 +68,6 @@
     <t>fhjfaosfjo</t>
   </si>
   <si>
-    <t>URL</t>
-  </si>
-  <si>
-    <t>https://demoapps.qspiders.com/ui?scenario=1</t>
-  </si>
-  <si>
     <t>Kanishk</t>
   </si>
   <si>
@@ -85,32 +76,72 @@
   <si>
     <t>gjgfea</t>
   </si>
+  <si>
+    <t>PlayWright</t>
+  </si>
+  <si>
+    <t>Java</t>
+  </si>
+  <si>
+    <t>Selenium</t>
+  </si>
+  <si>
+    <t>Cypress</t>
+  </si>
+  <si>
+    <t>WebDriverIO</t>
+  </si>
+  <si>
+    <t>EN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hello, sign in
+  Account &amp; Lists</t>
+  </si>
+  <si>
+    <t>Today's Deals</t>
+  </si>
+  <si>
+    <t>Gift Cards</t>
+  </si>
+  <si>
+    <t>Registry</t>
+  </si>
+  <si>
+    <t>Sell</t>
+  </si>
+  <si>
+    <t>Prime Video</t>
+  </si>
+  <si>
+    <t>Customer Service</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FFCE9178"/>
+      <family val="3"/>
+      <sz val="8"/>
+      <name val="Consolas"/>
     </font>
     <font>
       <u/>
-      <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FFCE9178"/>
-      <name val="Consolas"/>
-      <family val="3"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -130,19 +161,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -420,11 +449,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1">
         <v>35457</v>
       </c>
@@ -435,11 +464,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E9A5280-DCF3-4757-ACCD-A944F91358EF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -447,29 +476,29 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
       <c r="C3" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -478,46 +507,46 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92BAA13B-B3A0-47B6-B237-9803790C65FA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="D2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="1" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>15</v>
       </c>
       <c r="B3" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D3" t="s">
@@ -526,10 +555,97 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{A7A2A589-49C5-410E-8038-D90164A6F3A1}"/>
-    <hyperlink ref="C3" r:id="rId2" xr:uid="{700AED10-D075-48C0-8BEE-B12FB5342C19}"/>
+    <hyperlink ref="C2" r:id="rId1"/>
+    <hyperlink ref="C3" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>